<commit_message>
Add advanced paper browsing and hierarchy controls
</commit_message>
<xml_diff>
--- a/submit_template.xlsx
+++ b/submit_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22192" windowHeight="10455"/>
+    <workbookView windowWidth="30720" windowHeight="13500"/>
   </bookViews>
   <sheets>
     <sheet name="Papers" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>doi</t>
   </si>
@@ -84,66 +84,6 @@
   </si>
   <si>
     <t>notes</t>
-  </si>
-  <si>
-    <t>10.48550/arXiv.2407.07061</t>
-  </si>
-  <si>
-    <t>Internet of agents: Weaving a web of heterogeneous agents for collaborative intelligence</t>
-  </si>
-  <si>
-    <t>Weize Chen*, Ziming You*, Ran Li*, Yitong Guan*, Chen Qian, Chenyang Zhao Cheng Yang, Ruobing Xie, Zhiyuan Liu, Maosong Sun</t>
-  </si>
-  <si>
-    <t>2024-10-04</t>
-  </si>
-  <si>
-    <t>Base Techniques</t>
-  </si>
-  <si>
-    <t>先前的multi-agent系统的局限性，系统化平台化程度不足（缺乏第三方集成支持，无法分布式，通信协议和状态转换依赖于硬编码）</t>
-  </si>
-  <si>
-    <t>将互联网的开放、分布式、服务化思想引入，构建一种标准化、可扩展的支持分布式、异构的智能体集成与通信协议。</t>
-  </si>
-  <si>
-    <t>服务器：智能体注册（分发系统提示词）、管理已注册智能体（专家）、专家发现服务、群聊管理和消息传递；客户端：包装具体智能体，提供通信接口；三层结构；通信即可嵌套灵活群聊；群聊采用**有限状态机**管理流程；平台初始化与注册-&gt;任务触发团队形成-&gt;内部嵌套协作</t>
-  </si>
-  <si>
-    <t>在 GAIA 基准测试中，仅使用四个基础 ReAct 智能体即达到最佳性能；在 RAG 任务中，基于 GPT-3.5 的 IoA 达到或超过 GPT-4 的性能</t>
-  </si>
-  <si>
-    <t>实验中存在冗余消息，通信 Token 消耗增加近一倍，这证明agent作为对话者而非执行者的本质能力区别；单点服务器可能存在瓶颈；智能体通过注册获取提示词成为不同专家，仍高度依赖人工实验设计，且这种专家的能力是否可靠</t>
-  </si>
-  <si>
-    <t>https://openreview.net/forum?id=o1Et3MogPw</t>
-  </si>
-  <si>
-    <t>https://github.com/OpenBMB/IoA</t>
-  </si>
-  <si>
-    <t>The Thirteenth International Conference on Learning Representations</t>
-  </si>
-  <si>
-    <t>[AI generated] **智能体互联网：构建异构智能体网络以实现协同智能**
-**说明：**
-1.  **核心概念直译**：将 "Internet of Agents" 直译为“智能体互联网”，准确对应其借鉴互联网理念的核心创新，并与物联网（IoT）等术语形成概念类比，符合学术语境。
-2.  **副标题意译与优化**：将 "Weaving a web of heterogeneous agents for collaborative intelligence" 意译为“构建异构智能体网络</t>
-  </si>
-  <si>
-    <t>agent互联网，升级版ABM系统，采用类似互联网思想，C/S架构，分布化、服务化、平台化</t>
-  </si>
-  <si>
-    <t>figures/IoA.png;figures/IoA2.png</t>
-  </si>
-  <si>
-    <t>The rapid advancement of large language models (LLMs) has paved the way for the development of highly capable autonomous agents. However, existing multi-agent frameworks often struggle with integrating diverse capable third-party agents due to reliance on agents defined within their own ecosystems. They also face challenges in simulating distributed environments, as most frameworks are limited to single-device setups. Furthermore, these frameworks often rely on hard-coded communication pipelines, limiting their adaptability to dynamic task requirements. Inspired by the concept of the Internet, we propose the Internet of Agents (IoA), a novel framework that addresses these limitations by providing a flexible and scalable platform for LLM-based multi-agent collaboration. IoA introduces an agent integration protocol, an instant-messaging-like architecture design, and dynamic mechanisms for agent teaming and conversation flow control. Through extensive experiments on general assistant tasks, embodied AI tasks, and retrieval-augmented generation benchmarks, we demonstrate that IoA consistently outperforms state-of-the-art baselines, showcasing its ability to facilitate effective collaboration among heterogeneous agents. IoA represents a step towards linking diverse agents in an Internet-like environment, where agents can seamlessly collaborate to achieve greater intelligence and capabilities. We will release our code to facilitate further research.</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>每个agent被一个客户端包装；服务器不是agent，它只做四件事：注册、发现、建群、路由；相对于传统ABM，这是一个更大型的服务系统，该方法通过基于任务的“群聊”方式组织问题解决，相对传统回合制方式更加自由。本身也是一个高度可扩展系统。问题在于智能体通过注册获取提示词成为不同专家，仍依赖手工设计，且这种专家的能力是否可靠。对于社会模拟任务相对于传统方法有何决定性优势仍未可知</t>
   </si>
 </sst>
 </file>
@@ -156,14 +96,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -676,146 +609,146 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1163,7 +1096,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:X2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="5" width="15" customWidth="1"/>
     <col min="6" max="7" width="21" customWidth="1"/>
@@ -1235,74 +1168,30 @@
       </c>
     </row>
     <row r="2" s="1" customFormat="1" spans="1:24">
-      <c r="A2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
       <c r="T2" s="4"/>
-      <c r="U2" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="V2" s="4" t="s">
-        <v>36</v>
-      </c>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
       <c r="W2" s="4"/>
-      <c r="X2" s="4" t="s">
-        <v>36</v>
-      </c>
+      <c r="X2" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>